<commit_message>
Corrijo extraccion de edades y calculos de promedio y desviasion
</commit_message>
<xml_diff>
--- a/BdatosD_filtrado.xlsx
+++ b/BdatosD_filtrado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,20 +424,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>edad_min</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>edad_max</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>def_clas_edad</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>sexo_</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>aseguradora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>conducta</t>
         </is>
@@ -446,52 +456,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7  A 11</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>INFANCIA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>EPS COLSANITAS</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>HOSPITALIZACION PISO</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C3" t="n">
+        <v>59</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>NUEVA EPS</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -500,25 +522,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>29</v>
+      </c>
+      <c r="C4" t="n">
+        <v>59</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>COMPENSAR E.P.S.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -527,52 +555,64 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>29</v>
+      </c>
+      <c r="C5" t="n">
+        <v>59</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>COMPAÃ‘IA SURAMERICANA DE SERVICIOS DE SALUD S.A SUSALUD MEDICINA PREPAGADA</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>29 A 59</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NUEVA EPS</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -581,52 +621,64 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>COOMEVA E.P.S. S.A.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>HOSPITALIZACION PISO</t>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" t="n">
+        <v>60</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>PERSONA MAYOR</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FAMISANAR E.P.S. LTDA.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -635,25 +687,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>29</v>
+      </c>
+      <c r="C9" t="n">
+        <v>59</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -662,54 +720,66 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>29</v>
+      </c>
+      <c r="C10" t="n">
+        <v>59</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SALUDVIDA EPS S.A.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>60</v>
+      </c>
+      <c r="C11" t="n">
+        <v>60</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SANITAS E.P.S. S.A.</t>
+          <t>PERSONA MAYOR</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OBSERVACION</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
@@ -719,24 +789,30 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+      <c r="B12" t="n">
+        <v>29</v>
+      </c>
+      <c r="C12" t="n">
+        <v>59</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMPENSAR E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SANITAS E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OBSERVACION</t>
         </is>
       </c>
     </row>
@@ -746,76 +822,94 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B13" t="n">
+        <v>29</v>
+      </c>
+      <c r="C13" t="n">
+        <v>59</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>COMPAÃ‘IA SURAMERICANA DE SERVICIOS DE SALUD S.A SUSALUD MEDICINA PREPAGADA</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HOSPITALIZACION PISO</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ASOCIACION MUTUAL LA ESPERANZA ASMET SALUD ESS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>29</v>
+      </c>
+      <c r="C14" t="n">
+        <v>59</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>NUEVA EPS</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>OBSERVACION</t>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7  A 11</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>INFANCIA</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>29</v>
+      </c>
+      <c r="C15" t="n">
+        <v>59</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CAPRECOM EPS</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>COOMEVA E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -824,25 +918,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>60</v>
+      </c>
+      <c r="C16" t="n">
+        <v>60</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>COOMEVA E.P.S. S.A.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>POLICIA NACIONAL</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -851,54 +951,66 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>60</v>
+      </c>
+      <c r="C17" t="n">
+        <v>60</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>COOMEVA E.P.S. S.A.</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>HOSPITALIZACION PISO</t>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CAFESALUD E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>29</v>
+      </c>
+      <c r="C18" t="n">
+        <v>59</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
@@ -908,51 +1020,63 @@
           <t>60 Y MAS</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" t="n">
+        <v>60</v>
+      </c>
+      <c r="C19" t="n">
+        <v>60</v>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>PERSONA MAYOR</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>COOMEVA E.P.S. S.A.</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>FONDO DE PASIVO SOCIAL DE FERROCARRILES NACIONALES DE COLOMBIA.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OBSERVACION</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>29</v>
+      </c>
+      <c r="C20" t="n">
+        <v>59</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FAMISANAR E.P.S. LTDA.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ECOPETROL</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OBSERVACION</t>
         </is>
       </c>
     </row>
@@ -962,24 +1086,30 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B21" t="n">
+        <v>29</v>
+      </c>
+      <c r="C21" t="n">
+        <v>59</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NUEVA EPS</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CAJA DE PREVISION SOCIAL DE LA UNIVERSIDAD INDUSTRIAL DE SANTANDER CAPRUIS.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
@@ -989,49 +1119,61 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B22" t="n">
+        <v>29</v>
+      </c>
+      <c r="C22" t="n">
+        <v>59</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SALUDVIDA EPS S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>HOSPITALIZACION PISO</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0 A 6</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PRIMERA INFANCIA</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>29</v>
+      </c>
+      <c r="C23" t="n">
+        <v>59</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>COLPATRIA S.A MEDICINA PREPAGADA</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FIDUPREVISORA FONDO DE PRESTACIONES SOCIALES DEL MAGISTERIO</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1040,25 +1182,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0 A 6</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PRIMERA INFANCIA</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>29</v>
+      </c>
+      <c r="C24" t="n">
+        <v>59</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1067,25 +1215,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>29</v>
+      </c>
+      <c r="C25" t="n">
+        <v>59</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NO AFILIADO</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1094,52 +1248,64 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>60</v>
+      </c>
+      <c r="C26" t="n">
+        <v>60</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>PERSONA MAYOR</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>29</v>
+      </c>
+      <c r="C27" t="n">
+        <v>59</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>COOMEVA E.P.S. S.A.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1148,25 +1314,31 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>29</v>
+      </c>
+      <c r="C28" t="n">
+        <v>59</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>COOMEVA E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1178,24 +1350,30 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B29" t="n">
+        <v>29</v>
+      </c>
+      <c r="C29" t="n">
+        <v>59</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SANITAS E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OBSERVACION</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
@@ -1205,22 +1383,28 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="n">
+        <v>59</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ASOCIACION MUTUAL LA ESPERANZA ASMET SALUD ESS</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1229,25 +1413,31 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>29</v>
+      </c>
+      <c r="C31" t="n">
+        <v>59</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>FAMISANAR E.P.S. LTDA.</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
         <is>
           <t>HOSPITALIZACION PISO</t>
         </is>
@@ -1256,106 +1446,130 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>29</v>
+      </c>
+      <c r="C32" t="n">
+        <v>59</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OBSERVACION</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0 A 6</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>PRIMERA INFANCIA</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>29</v>
+      </c>
+      <c r="C33" t="n">
+        <v>59</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>NUEVA EPS</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>HOSPITALIZACION PISO</t>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CAFESALUD E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>60</v>
+      </c>
+      <c r="C34" t="n">
+        <v>60</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>FAMISANAR E.P.S. LTDA.</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>OBSERVACION</t>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>29</v>
+      </c>
+      <c r="C35" t="n">
+        <v>59</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SANITAS E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1364,25 +1578,31 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>29 A 59</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>60</v>
+      </c>
+      <c r="C36" t="n">
+        <v>60</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>PERSONA MAYOR</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1394,22 +1614,28 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B37" t="n">
+        <v>29</v>
+      </c>
+      <c r="C37" t="n">
+        <v>59</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>COOMEVA E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>CAPRECOM EPS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1418,52 +1644,64 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0 A 6</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>PRIMERA INFANCIA</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>29</v>
+      </c>
+      <c r="C38" t="n">
+        <v>59</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SALUD TOTAL S.A. E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AMBULATORIA</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>COOSALUD ESS EPS-S</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>HOSPITALIZACION PISO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0 A 6</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>PRIMERA INFANCIA</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>29</v>
+      </c>
+      <c r="C39" t="n">
+        <v>59</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>COOMEVA E.P.S. S.A.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1472,25 +1710,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>29</v>
+      </c>
+      <c r="C40" t="n">
+        <v>59</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>COOMEVA E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1499,25 +1743,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>29</v>
+      </c>
+      <c r="C41" t="n">
+        <v>59</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>NUEVA EPS</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1526,25 +1776,31 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>29</v>
+      </c>
+      <c r="C42" t="n">
+        <v>59</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>POLICIA NACIONAL</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1553,25 +1809,31 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>29</v>
+      </c>
+      <c r="C43" t="n">
+        <v>59</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ADULTEZ</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>CAFESALUD E.P.S. S.A.</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1583,76 +1845,94 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+      <c r="B44" t="n">
+        <v>29</v>
+      </c>
+      <c r="C44" t="n">
+        <v>59</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>NUEVA EPS</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HOSPITALIZACION PISO</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>60 Y MAS</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>PERSONA MAYOR</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>29</v>
+      </c>
+      <c r="C45" t="n">
+        <v>59</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FONDO DE PASIVO SOCIAL DE FERROCARRILES NACIONALES DE COLOMBIA.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OBSERVACION</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>29</v>
+      </c>
+      <c r="C46" t="n">
+        <v>59</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SALUDCOOP E.P.S.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1661,25 +1941,31 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>18 A 28</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>JOVENES</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>29</v>
+      </c>
+      <c r="C47" t="n">
+        <v>59</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SANITAS E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SALUDCOOP E.P.S.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1688,25 +1974,31 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7  A 11</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>INFANCIA</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>29</v>
+      </c>
+      <c r="C48" t="n">
+        <v>59</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>COOMEVA E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>SANITAS E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1715,25 +2007,31 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
+          <t>29 A 59</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>29</v>
+      </c>
+      <c r="C49" t="n">
+        <v>59</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>COOMEVA E.P.S. S.A.</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SALUD TOTAL S.A. E.P.S.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1742,25 +2040,31 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>12 A 17</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
+          <t>60 Y MAS</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>60</v>
+      </c>
+      <c r="C50" t="n">
+        <v>60</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>PERSONA MAYOR</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>SALUDCOOP E.P.S.</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>NUEVA EPS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
         <is>
           <t>AMBULATORIA</t>
         </is>
@@ -1772,24 +2076,30 @@
           <t>29 A 59</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>ADULTEZ</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+      <c r="B51" t="n">
+        <v>29</v>
+      </c>
+      <c r="C51" t="n">
+        <v>59</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ECOPETROL</t>
+          <t>ADULTEZ</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OBSERVACION</t>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>COOMEVA E.P.S. S.A.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>AMBULATORIA</t>
         </is>
       </c>
     </row>

</xml_diff>